<commit_message>
update  code. Add dataset_loader.ipynb,evaluate_ft_model.ipynb,rag.ipynb
</commit_message>
<xml_diff>
--- a/writings/Paper_Screening.xlsx
+++ b/writings/Paper_Screening.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\COMP9800\github\gradproj\writings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381B5C66-63B5-4242-A19A-5B085D6C78F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7493439-1286-41C6-968F-47929715C811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="337" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="337" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="665">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="669">
   <si>
     <t>Title</t>
   </si>
@@ -2869,6 +2869,22 @@
   </si>
   <si>
     <t>Classification evaluation metrics for a variety of datasets</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pogorelov, Konstantin, Kristin Ranheim Randel, Carsten Griwodz, et al. “KVASIR: A Multi-Class Image Dataset for Computer Aided Gastrointestinal Disease Detection.” Proceedings of the 8th ACM on Multimedia Systems Conference, ACM, June 20, 2017, 164–69. https://doi.org/10.1145/3083187.3083212.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kvasir Dataset</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Song, Yiming, Zhengjie Zhang, Ruilan Wang, et al. “CAS-Colon: A Comprehensive Colonoscopy Anatomical Segmentation Dataset for Artificial Intelligence Development.” Scientific Data 12 (August 2025): 1382. https://doi.org/10.1038/s41597-025-05588-3.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CAS-COLON</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -5201,7 +5217,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="100.8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" ht="100.8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>98</v>
       </c>
@@ -5255,7 +5271,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="86.4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" ht="86.4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>98</v>
       </c>
@@ -5309,7 +5325,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="100.8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" ht="100.8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>98</v>
       </c>
@@ -5363,7 +5379,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="86.4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" ht="86.4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>98</v>
       </c>
@@ -5417,7 +5433,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="158.4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" ht="158.4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>98</v>
       </c>
@@ -5474,7 +5490,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="86.4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" ht="86.4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>98</v>
       </c>
@@ -5577,7 +5593,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="144" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" ht="144" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>98</v>
       </c>
@@ -5631,7 +5647,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="100.8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" ht="100.8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>98</v>
       </c>
@@ -5688,7 +5704,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="43" spans="1:20" ht="87" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" ht="87" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>98</v>
       </c>
@@ -5745,7 +5761,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="86.4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" ht="86.4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>98</v>
       </c>
@@ -5799,7 +5815,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="86.4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" ht="86.4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>98</v>
       </c>
@@ -5856,7 +5872,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="100.8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" ht="100.8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>338</v>
       </c>
@@ -7489,7 +7505,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:20" ht="86.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:20" ht="86.4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>99</v>
       </c>
@@ -7515,7 +7531,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="82" spans="1:20" ht="86.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:20" ht="86.4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>99</v>
       </c>
@@ -7538,7 +7554,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="83" spans="1:20" ht="115.2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:20" ht="115.2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>99</v>
       </c>
@@ -7561,7 +7577,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="84" spans="1:20" ht="86.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:20" ht="86.4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>99</v>
       </c>
@@ -7584,7 +7600,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="85" spans="1:20" ht="158.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:20" ht="158.4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>99</v>
       </c>
@@ -7607,7 +7623,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="86" spans="1:20" ht="86.4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:20" ht="86.4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>99</v>
       </c>
@@ -7630,7 +7646,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="87" spans="1:20" ht="72" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:20" ht="72" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>99</v>
       </c>
@@ -7653,7 +7669,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="88" spans="1:20" ht="72" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:20" ht="72" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>99</v>
       </c>
@@ -8189,13 +8205,8 @@
   <autoFilter ref="A1:T99" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="TTI"/>
+        <filter val="Dataset"/>
       </filters>
-    </filterColumn>
-    <filterColumn colId="1">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
     </filterColumn>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A34:T93">
@@ -8209,7 +8220,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84EF80BE-0DA4-44B6-8D40-C8D0EF1A7933}">
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.77734375" style="1" customWidth="1"/>
@@ -9092,7 +9103,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="65" spans="1:2" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -9100,12 +9111,34 @@
         <v>631</v>
       </c>
     </row>
-    <row r="66" spans="1:2" ht="158.4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" ht="158.4" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>633</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="129.6" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>66</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>665</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="115.2" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>67</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>667</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>